<commit_message>
Files for calculate insurance project added
</commit_message>
<xml_diff>
--- a/testdata/TestOutputData.xlsx
+++ b/testdata/TestOutputData.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" r:id="rId1" sheetId="1"/>
-    <sheet name="home_loan" r:id="rId8" sheetId="24"/>
-    <sheet name="car_loan" r:id="rId9" sheetId="25"/>
-    <sheet name="emi_calculator" r:id="rId10" sheetId="26"/>
+    <sheet name="home_loan" r:id="rId8" sheetId="35"/>
+    <sheet name="car_loan" r:id="rId9" sheetId="36"/>
+    <sheet name="emi_calculator" r:id="rId10" sheetId="37"/>
   </sheets>
   <calcPr calcId="0"/>
   <oleSize ref="A1:N11"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="42">
   <si>
     <t>abc</t>
   </si>
@@ -105,6 +105,54 @@
   </si>
   <si>
     <t>₹ 0.00</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>₹ 9,84,149</t>
+  </si>
+  <si>
+    <t>₹ 68,053</t>
+  </si>
+  <si>
+    <t>₹ 10,52,202</t>
+  </si>
+  <si>
+    <t>₹ 5,15,851</t>
+  </si>
+  <si>
+    <t>65.61%</t>
+  </si>
+  <si>
+    <t>2027</t>
+  </si>
+  <si>
+    <t>₹ 10,250</t>
+  </si>
+  <si>
+    <t>₹ 5,26,101</t>
+  </si>
+  <si>
+    <t>₹ 9,84,148.76</t>
+  </si>
+  <si>
+    <t>₹ 68,053.40</t>
+  </si>
+  <si>
+    <t>₹ 10,52,202.16</t>
+  </si>
+  <si>
+    <t>₹ 5,15,851.24</t>
+  </si>
+  <si>
+    <t>₹ 5,15,851.27</t>
+  </si>
+  <si>
+    <t>₹ 10,249.81</t>
+  </si>
+  <si>
+    <t>₹ 5,26,101.08</t>
   </si>
 </sst>
 </file>
@@ -141,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="451">
+  <cellXfs count="649">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
     <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1488,6 +1536,600 @@
       <alignment wrapText="true"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -1807,11 +2449,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
     </row>
@@ -1820,76 +2462,76 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.49609375" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.55078125" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.7734375" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.9921875" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="10.4375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.14453125" collapsed="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.9296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.359375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.8671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.55078125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.359375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.37890625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="397" t="s">
+      <c r="A1" s="595" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="398" t="s">
+      <c r="B1" s="596" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="399" t="s">
+      <c r="C1" s="597" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="400" t="s">
+      <c r="D1" s="598" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="401" t="s">
+      <c r="E1" s="599" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="402" t="s">
+      <c r="F1" s="600" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="403" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="404" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="405" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="406" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="407" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="408" t="s">
-        <v>12</v>
+      <c r="A2" s="601" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="602" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="603" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="604" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="605" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="606" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="409" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="410" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="411" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="412" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="413" t="s">
+      <c r="A3" s="607" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="608" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="609" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="610" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="611" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="414" t="s">
+      <c r="F3" s="612" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1898,76 +2540,76 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.49609375" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="11.55078125" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="8.7734375" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="13.9921875" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="10.4375" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.14453125" collapsed="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.9296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="9.359375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="7.8671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.55078125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="9.359375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.37890625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="415" t="s">
+      <c r="A1" s="613" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="416" t="s">
+      <c r="B1" s="614" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="417" t="s">
+      <c r="C1" s="615" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="418" t="s">
+      <c r="D1" s="616" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="419" t="s">
+      <c r="E1" s="617" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="420" t="s">
+      <c r="F1" s="618" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="421" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="422" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="423" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="424" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="425" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="426" t="s">
-        <v>12</v>
+      <c r="A2" s="619" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="620" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="621" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="622" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="623" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="624" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="427" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="428" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="429" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="430" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="431" t="s">
+      <c r="A3" s="625" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="626" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="627" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="628" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="629" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="432" t="s">
+      <c r="F3" s="630" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1976,76 +2618,76 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.49609375" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="14.3359375" collapsed="true"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.55859375" collapsed="true"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="14.3359375" collapsed="true"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="13.22265625" collapsed="true"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="17.14453125" collapsed="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.9296875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="11.859375"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="10.3671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.859375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="11.859375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="15.37890625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="433" t="s">
+      <c r="A1" s="631" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="434" t="s">
+      <c r="B1" s="632" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="435" t="s">
+      <c r="C1" s="633" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="436" t="s">
+      <c r="D1" s="634" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="437" t="s">
+      <c r="E1" s="635" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="438" t="s">
+      <c r="F1" s="636" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="439" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="440" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="441" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="442" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="443" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="444" t="s">
-        <v>12</v>
+      <c r="A2" s="637" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="638" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="639" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="640" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="641" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="642" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="445" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="446" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="447" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="448" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="449" t="s">
+      <c r="A3" s="643" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="644" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="645" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="646" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="647" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="450" t="s">
+      <c r="F3" s="648" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>